<commit_message>
Metamorfosis V2.0: Glassmorphism Elite, Live Sync Fixes & Estetica Command Center
</commit_message>
<xml_diff>
--- a/MAPA CPAG/lotesv CPAG.xlsx
+++ b/MAPA CPAG/lotesv CPAG.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d9d62b85ef481923/Escritorio/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://vbcrd.sharepoint.com/sites/VBCRD/Shared Documents/IDMP/VBC2/Informes Fideicomiso VBC/Presentacion Paliza diciembre 2025/Mapa/MAPA CPAG/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="106" documentId="8_{87FD73C8-A84B-4DB9-A172-7824E412B364}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5B66D906-56CC-44E7-9743-5A8CB8E4A833}"/>
+  <xr:revisionPtr revIDLastSave="112" documentId="8_{87FD73C8-A84B-4DB9-A172-7824E412B364}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EB8233A6-596C-491F-A559-36CBBCFBDE23}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="5832" yWindow="3348" windowWidth="17208" windowHeight="8892" xr2:uid="{AEF7EA20-191D-44D4-A8BF-F71162BE4BC3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{AEF7EA20-191D-44D4-A8BF-F71162BE4BC3}"/>
   </bookViews>
   <sheets>
     <sheet name="lotesv2" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" calcCompleted="0"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -338,249 +338,6 @@
     <t>INSTITUCIONAL</t>
   </si>
   <si>
-    <t>469.056 m²</t>
-  </si>
-  <si>
-    <t>1,002.649 m²</t>
-  </si>
-  <si>
-    <t>1,321.491 m²</t>
-  </si>
-  <si>
-    <t>3,005.287 m²</t>
-  </si>
-  <si>
-    <t>3,186.243 m²</t>
-  </si>
-  <si>
-    <t>1,033.456 m²</t>
-  </si>
-  <si>
-    <t>1,133.952 m²</t>
-  </si>
-  <si>
-    <t>1,162.884 m²</t>
-  </si>
-  <si>
-    <t>1,168.106 m²</t>
-  </si>
-  <si>
-    <t>1,176.709 m²</t>
-  </si>
-  <si>
-    <t>1,219.906 m²</t>
-  </si>
-  <si>
-    <t>1,258.031 m²</t>
-  </si>
-  <si>
-    <t>1,288.575 m²</t>
-  </si>
-  <si>
-    <t>1,462.184 m²</t>
-  </si>
-  <si>
-    <t>1,593.489 m²</t>
-  </si>
-  <si>
-    <t>1,706.054 m²</t>
-  </si>
-  <si>
-    <t>1,720.259 m²</t>
-  </si>
-  <si>
-    <t>1,724.180 m²</t>
-  </si>
-  <si>
-    <t>1,758.331 m²</t>
-  </si>
-  <si>
-    <t>1,849.741 m²</t>
-  </si>
-  <si>
-    <t>1,945.897 m²</t>
-  </si>
-  <si>
-    <t>2,069.560 m²</t>
-  </si>
-  <si>
-    <t>2,210.760 m²</t>
-  </si>
-  <si>
-    <t>2,636.790 m²</t>
-  </si>
-  <si>
-    <t>2,708.916 m²</t>
-  </si>
-  <si>
-    <t>7,004.929 m²</t>
-  </si>
-  <si>
-    <t>10,215.880 m²</t>
-  </si>
-  <si>
-    <t>10,271.238 m²</t>
-  </si>
-  <si>
-    <t>10,364.996 m²</t>
-  </si>
-  <si>
-    <t>10,579.592 m²</t>
-  </si>
-  <si>
-    <t>11,184.263 m²</t>
-  </si>
-  <si>
-    <t>12,221.872 m²</t>
-  </si>
-  <si>
-    <t>12,328.505 m²</t>
-  </si>
-  <si>
-    <t>12,756.993 m²</t>
-  </si>
-  <si>
-    <t>13,359.217 m²</t>
-  </si>
-  <si>
-    <t>13,479.100 m²</t>
-  </si>
-  <si>
-    <t>14,004.129 m²</t>
-  </si>
-  <si>
-    <t>14,152.002 m²</t>
-  </si>
-  <si>
-    <t>14,212.071 m²</t>
-  </si>
-  <si>
-    <t>14,262.965 m²</t>
-  </si>
-  <si>
-    <t>14,344.217 m²</t>
-  </si>
-  <si>
-    <t>14,496.632 m²</t>
-  </si>
-  <si>
-    <t>15,235.223 m²</t>
-  </si>
-  <si>
-    <t>15,304.096 m²</t>
-  </si>
-  <si>
-    <t>15,305.861 m²</t>
-  </si>
-  <si>
-    <t>15,337.539 m²</t>
-  </si>
-  <si>
-    <t>15,424.655 m²</t>
-  </si>
-  <si>
-    <t>15,852.345 m²</t>
-  </si>
-  <si>
-    <t>16,273.832 m²</t>
-  </si>
-  <si>
-    <t>16,449.123 m²</t>
-  </si>
-  <si>
-    <t>16,732.601 m²</t>
-  </si>
-  <si>
-    <t>17,110.400 m²</t>
-  </si>
-  <si>
-    <t>18,781.390 m²</t>
-  </si>
-  <si>
-    <t>19,433.392 m²</t>
-  </si>
-  <si>
-    <t>20,057.607 m²</t>
-  </si>
-  <si>
-    <t>23,162.823 m²</t>
-  </si>
-  <si>
-    <t>24,280.757 m²</t>
-  </si>
-  <si>
-    <t>686.446 m²</t>
-  </si>
-  <si>
-    <t>923.260 m²</t>
-  </si>
-  <si>
-    <t>924.590 m²</t>
-  </si>
-  <si>
-    <t>1,196.249 m²</t>
-  </si>
-  <si>
-    <t>1,561.283 m²</t>
-  </si>
-  <si>
-    <t>1,593.125 m²</t>
-  </si>
-  <si>
-    <t>1,594.628 m²</t>
-  </si>
-  <si>
-    <t>1,642.509 m²</t>
-  </si>
-  <si>
-    <t>1,925.404 m²</t>
-  </si>
-  <si>
-    <t>1,970.665 m²</t>
-  </si>
-  <si>
-    <t>2,004.156 m²</t>
-  </si>
-  <si>
-    <t>2,130.360 m²</t>
-  </si>
-  <si>
-    <t>2,432.208 m²</t>
-  </si>
-  <si>
-    <t>3,046.704 m²</t>
-  </si>
-  <si>
-    <t>3,378.323 m²</t>
-  </si>
-  <si>
-    <t>3,860.101 m²</t>
-  </si>
-  <si>
-    <t>4,732.365 m²</t>
-  </si>
-  <si>
-    <t>4,952.633 m²</t>
-  </si>
-  <si>
-    <t>5,051.997 m²</t>
-  </si>
-  <si>
-    <t>9,010.227 m²</t>
-  </si>
-  <si>
-    <t>9,667.620 m²</t>
-  </si>
-  <si>
-    <t>9,825.978 m²</t>
-  </si>
-  <si>
-    <t>11,042.007 m²</t>
-  </si>
-  <si>
-    <t>20,698.670 m²</t>
-  </si>
-  <si>
     <t>C-01</t>
   </si>
   <si>
@@ -635,52 +392,295 @@
     <t>INFRAESTRUCTURA</t>
   </si>
   <si>
-    <t>49,976.951 m²</t>
-  </si>
-  <si>
-    <t>2,300.918 m²</t>
-  </si>
-  <si>
-    <t>6,688.925 m²</t>
-  </si>
-  <si>
-    <t>2,415.205 m²</t>
-  </si>
-  <si>
-    <t>3,480.806 m²</t>
-  </si>
-  <si>
-    <t>2,290.665 m²</t>
-  </si>
-  <si>
-    <t>3,745.477 m²</t>
-  </si>
-  <si>
-    <t>2,118.224 m²</t>
-  </si>
-  <si>
-    <t>1,724.711 m²</t>
-  </si>
-  <si>
-    <t>3,961.132 m²</t>
-  </si>
-  <si>
-    <t>3,085.302 m²</t>
-  </si>
-  <si>
-    <t>17,863.494 m²</t>
-  </si>
-  <si>
-    <t>2,674.373 m²</t>
-  </si>
-  <si>
-    <t>664.668 m²</t>
-  </si>
-  <si>
-    <t>897.490 m²</t>
-  </si>
-  <si>
-    <t>917.339 m²</t>
+    <t>469.056</t>
+  </si>
+  <si>
+    <t>1,002.649</t>
+  </si>
+  <si>
+    <t>1,321.491</t>
+  </si>
+  <si>
+    <t>3,005.287</t>
+  </si>
+  <si>
+    <t>3,186.243</t>
+  </si>
+  <si>
+    <t>1,033.456</t>
+  </si>
+  <si>
+    <t>1,133.952</t>
+  </si>
+  <si>
+    <t>1,162.884</t>
+  </si>
+  <si>
+    <t>1,168.106</t>
+  </si>
+  <si>
+    <t>1,176.709</t>
+  </si>
+  <si>
+    <t>1,219.906</t>
+  </si>
+  <si>
+    <t>1,258.031</t>
+  </si>
+  <si>
+    <t>1,288.575</t>
+  </si>
+  <si>
+    <t>1,462.184</t>
+  </si>
+  <si>
+    <t>1,593.489</t>
+  </si>
+  <si>
+    <t>1,706.054</t>
+  </si>
+  <si>
+    <t>1,720.259</t>
+  </si>
+  <si>
+    <t>1,724.180</t>
+  </si>
+  <si>
+    <t>1,758.331</t>
+  </si>
+  <si>
+    <t>1,849.741</t>
+  </si>
+  <si>
+    <t>1,945.897</t>
+  </si>
+  <si>
+    <t>2,069.560</t>
+  </si>
+  <si>
+    <t>2,210.760</t>
+  </si>
+  <si>
+    <t>2,636.790</t>
+  </si>
+  <si>
+    <t>2,708.916</t>
+  </si>
+  <si>
+    <t>7,004.929</t>
+  </si>
+  <si>
+    <t>10,215.880</t>
+  </si>
+  <si>
+    <t>10,271.238</t>
+  </si>
+  <si>
+    <t>10,364.996</t>
+  </si>
+  <si>
+    <t>10,579.592</t>
+  </si>
+  <si>
+    <t>11,184.263</t>
+  </si>
+  <si>
+    <t>12,221.872</t>
+  </si>
+  <si>
+    <t>12,328.505</t>
+  </si>
+  <si>
+    <t>12,756.993</t>
+  </si>
+  <si>
+    <t>13,359.217</t>
+  </si>
+  <si>
+    <t>13,479.100</t>
+  </si>
+  <si>
+    <t>14,004.129</t>
+  </si>
+  <si>
+    <t>14,152.002</t>
+  </si>
+  <si>
+    <t>14,212.071</t>
+  </si>
+  <si>
+    <t>14,262.965</t>
+  </si>
+  <si>
+    <t>14,344.217</t>
+  </si>
+  <si>
+    <t>14,496.632</t>
+  </si>
+  <si>
+    <t>15,235.223</t>
+  </si>
+  <si>
+    <t>15,304.096</t>
+  </si>
+  <si>
+    <t>15,305.861</t>
+  </si>
+  <si>
+    <t>15,337.539</t>
+  </si>
+  <si>
+    <t>15,424.655</t>
+  </si>
+  <si>
+    <t>15,852.345</t>
+  </si>
+  <si>
+    <t>16,273.832</t>
+  </si>
+  <si>
+    <t>16,449.123</t>
+  </si>
+  <si>
+    <t>16,732.601</t>
+  </si>
+  <si>
+    <t>17,110.400</t>
+  </si>
+  <si>
+    <t>18,781.390</t>
+  </si>
+  <si>
+    <t>19,433.392</t>
+  </si>
+  <si>
+    <t>20,057.607</t>
+  </si>
+  <si>
+    <t>23,162.823</t>
+  </si>
+  <si>
+    <t>24,280.757</t>
+  </si>
+  <si>
+    <t>686.446</t>
+  </si>
+  <si>
+    <t>923.260</t>
+  </si>
+  <si>
+    <t>924.590</t>
+  </si>
+  <si>
+    <t>1,196.249</t>
+  </si>
+  <si>
+    <t>1,561.283</t>
+  </si>
+  <si>
+    <t>1,593.125</t>
+  </si>
+  <si>
+    <t>1,594.628</t>
+  </si>
+  <si>
+    <t>1,642.509</t>
+  </si>
+  <si>
+    <t>1,925.404</t>
+  </si>
+  <si>
+    <t>1,970.665</t>
+  </si>
+  <si>
+    <t>2,004.156</t>
+  </si>
+  <si>
+    <t>2,130.360</t>
+  </si>
+  <si>
+    <t>2,432.208</t>
+  </si>
+  <si>
+    <t>3,046.704</t>
+  </si>
+  <si>
+    <t>3,378.323</t>
+  </si>
+  <si>
+    <t>3,860.101</t>
+  </si>
+  <si>
+    <t>4,732.365</t>
+  </si>
+  <si>
+    <t>4,952.633</t>
+  </si>
+  <si>
+    <t>5,051.997</t>
+  </si>
+  <si>
+    <t>9,010.227</t>
+  </si>
+  <si>
+    <t>9,667.620</t>
+  </si>
+  <si>
+    <t>9,825.978</t>
+  </si>
+  <si>
+    <t>11,042.007</t>
+  </si>
+  <si>
+    <t>20,698.670</t>
+  </si>
+  <si>
+    <t>49,976.951</t>
+  </si>
+  <si>
+    <t>2,300.918</t>
+  </si>
+  <si>
+    <t>6,688.925</t>
+  </si>
+  <si>
+    <t>2,415.205</t>
+  </si>
+  <si>
+    <t>3,480.806</t>
+  </si>
+  <si>
+    <t>2,290.665</t>
+  </si>
+  <si>
+    <t>3,745.477</t>
+  </si>
+  <si>
+    <t>2,118.224</t>
+  </si>
+  <si>
+    <t>1,724.711</t>
+  </si>
+  <si>
+    <t>3,961.132</t>
+  </si>
+  <si>
+    <t>3,085.302</t>
+  </si>
+  <si>
+    <t>17,863.494</t>
+  </si>
+  <si>
+    <t>2,674.373</t>
+  </si>
+  <si>
+    <t>664.668</t>
+  </si>
+  <si>
+    <t>897.490</t>
+  </si>
+  <si>
+    <t>917.339</t>
   </si>
 </sst>
 </file>
@@ -1171,52 +1171,52 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
-    <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20% - Énfasis2" xfId="23" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20% - Énfasis3" xfId="27" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20% - Énfasis4" xfId="31" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20% - Énfasis5" xfId="35" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20% - Énfasis6" xfId="39" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis1" xfId="20" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis2" xfId="24" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis3" xfId="28" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis4" xfId="32" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis5" xfId="36" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis6" xfId="40" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis1" xfId="21" builtinId="32" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis2" xfId="25" builtinId="36" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis3" xfId="29" builtinId="40" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis4" xfId="33" builtinId="44" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis5" xfId="37" builtinId="48" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis6" xfId="41" builtinId="52" customBuiltin="1"/>
-    <cellStyle name="Bueno" xfId="6" builtinId="26" customBuiltin="1"/>
-    <cellStyle name="Cálculo" xfId="11" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="Celda de comprobación" xfId="13" builtinId="23" customBuiltin="1"/>
-    <cellStyle name="Celda vinculada" xfId="12" builtinId="24" customBuiltin="1"/>
-    <cellStyle name="Encabezado 1" xfId="2" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="Encabezado 4" xfId="5" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="Énfasis1" xfId="18" builtinId="29" customBuiltin="1"/>
-    <cellStyle name="Énfasis2" xfId="22" builtinId="33" customBuiltin="1"/>
-    <cellStyle name="Énfasis3" xfId="26" builtinId="37" customBuiltin="1"/>
-    <cellStyle name="Énfasis4" xfId="30" builtinId="41" customBuiltin="1"/>
-    <cellStyle name="Énfasis5" xfId="34" builtinId="45" customBuiltin="1"/>
-    <cellStyle name="Énfasis6" xfId="38" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="Entrada" xfId="9" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="Incorrecto" xfId="7" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
+    <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
+    <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
+    <cellStyle name="20% - Accent4" xfId="31" builtinId="42" customBuiltin="1"/>
+    <cellStyle name="20% - Accent5" xfId="35" builtinId="46" customBuiltin="1"/>
+    <cellStyle name="20% - Accent6" xfId="39" builtinId="50" customBuiltin="1"/>
+    <cellStyle name="40% - Accent1" xfId="20" builtinId="31" customBuiltin="1"/>
+    <cellStyle name="40% - Accent2" xfId="24" builtinId="35" customBuiltin="1"/>
+    <cellStyle name="40% - Accent3" xfId="28" builtinId="39" customBuiltin="1"/>
+    <cellStyle name="40% - Accent4" xfId="32" builtinId="43" customBuiltin="1"/>
+    <cellStyle name="40% - Accent5" xfId="36" builtinId="47" customBuiltin="1"/>
+    <cellStyle name="40% - Accent6" xfId="40" builtinId="51" customBuiltin="1"/>
+    <cellStyle name="60% - Accent1" xfId="21" builtinId="32" customBuiltin="1"/>
+    <cellStyle name="60% - Accent2" xfId="25" builtinId="36" customBuiltin="1"/>
+    <cellStyle name="60% - Accent3" xfId="29" builtinId="40" customBuiltin="1"/>
+    <cellStyle name="60% - Accent4" xfId="33" builtinId="44" customBuiltin="1"/>
+    <cellStyle name="60% - Accent5" xfId="37" builtinId="48" customBuiltin="1"/>
+    <cellStyle name="60% - Accent6" xfId="41" builtinId="52" customBuiltin="1"/>
+    <cellStyle name="Accent1" xfId="18" builtinId="29" customBuiltin="1"/>
+    <cellStyle name="Accent2" xfId="22" builtinId="33" customBuiltin="1"/>
+    <cellStyle name="Accent3" xfId="26" builtinId="37" customBuiltin="1"/>
+    <cellStyle name="Accent4" xfId="30" builtinId="41" customBuiltin="1"/>
+    <cellStyle name="Accent5" xfId="34" builtinId="45" customBuiltin="1"/>
+    <cellStyle name="Accent6" xfId="38" builtinId="49" customBuiltin="1"/>
+    <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="Explanatory Text" xfId="16" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
+    <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
     <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Notas" xfId="15" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="Salida" xfId="10" builtinId="21" customBuiltin="1"/>
-    <cellStyle name="Texto de advertencia" xfId="14" builtinId="11" customBuiltin="1"/>
-    <cellStyle name="Texto explicativo" xfId="16" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Título" xfId="1" builtinId="15" customBuiltin="1"/>
-    <cellStyle name="Título 2" xfId="3" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="Título 3" xfId="4" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Note" xfId="15" builtinId="10" customBuiltin="1"/>
+    <cellStyle name="Output" xfId="10" builtinId="21" customBuiltin="1"/>
+    <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
+    <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="2">
     <dxf>
-      <numFmt numFmtId="19" formatCode="d/m/yyyy"/>
+      <numFmt numFmtId="164" formatCode="d/m/yyyy"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -1232,10 +1232,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1264,7 +1260,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1581,10 +1577,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{796055CF-22E4-4820-BA67-C984C73675DB}">
   <dimension ref="A1:P99"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.21875" style="3" customWidth="1"/>
+    <col min="2" max="2" width="16.88671875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.109375" customWidth="1"/>
+    <col min="7" max="7" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="19.109375" customWidth="1"/>
     <col min="11" max="11" width="14.44140625" customWidth="1"/>
     <col min="12" max="12" width="12.21875" customWidth="1"/>
@@ -1650,7 +1648,7 @@
         <v>97</v>
       </c>
       <c r="G2" t="s">
-        <v>101</v>
+        <v>119</v>
       </c>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
@@ -1663,7 +1661,7 @@
         <v>97</v>
       </c>
       <c r="G3" t="s">
-        <v>102</v>
+        <v>120</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.3">
@@ -1674,7 +1672,7 @@
         <v>97</v>
       </c>
       <c r="G4" t="s">
-        <v>103</v>
+        <v>121</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.3">
@@ -1685,7 +1683,7 @@
         <v>97</v>
       </c>
       <c r="G5" t="s">
-        <v>104</v>
+        <v>122</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.3">
@@ -1696,7 +1694,7 @@
         <v>97</v>
       </c>
       <c r="G6" t="s">
-        <v>105</v>
+        <v>123</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.3">
@@ -1707,7 +1705,7 @@
         <v>98</v>
       </c>
       <c r="G7" t="s">
-        <v>106</v>
+        <v>124</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.3">
@@ -1718,7 +1716,7 @@
         <v>98</v>
       </c>
       <c r="G8" t="s">
-        <v>107</v>
+        <v>125</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.3">
@@ -1729,7 +1727,7 @@
         <v>98</v>
       </c>
       <c r="G9" t="s">
-        <v>108</v>
+        <v>126</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.3">
@@ -1740,7 +1738,7 @@
         <v>98</v>
       </c>
       <c r="G10" t="s">
-        <v>109</v>
+        <v>127</v>
       </c>
       <c r="K10" s="1"/>
     </row>
@@ -1752,7 +1750,7 @@
         <v>98</v>
       </c>
       <c r="G11" t="s">
-        <v>110</v>
+        <v>128</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.3">
@@ -1763,7 +1761,7 @@
         <v>98</v>
       </c>
       <c r="G12" t="s">
-        <v>111</v>
+        <v>129</v>
       </c>
       <c r="J12" s="1"/>
     </row>
@@ -1775,7 +1773,7 @@
         <v>98</v>
       </c>
       <c r="G13" t="s">
-        <v>112</v>
+        <v>130</v>
       </c>
       <c r="K13" s="1"/>
     </row>
@@ -1787,7 +1785,7 @@
         <v>98</v>
       </c>
       <c r="G14" t="s">
-        <v>113</v>
+        <v>131</v>
       </c>
       <c r="K14" s="1"/>
     </row>
@@ -1799,7 +1797,7 @@
         <v>98</v>
       </c>
       <c r="G15" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.3">
@@ -1810,7 +1808,7 @@
         <v>98</v>
       </c>
       <c r="G16" t="s">
-        <v>115</v>
+        <v>133</v>
       </c>
       <c r="J16" s="1"/>
       <c r="K16" s="1"/>
@@ -1823,7 +1821,7 @@
         <v>98</v>
       </c>
       <c r="G17" t="s">
-        <v>116</v>
+        <v>134</v>
       </c>
       <c r="K17" s="1"/>
     </row>
@@ -1835,7 +1833,7 @@
         <v>98</v>
       </c>
       <c r="G18" t="s">
-        <v>117</v>
+        <v>135</v>
       </c>
       <c r="K18" s="1"/>
     </row>
@@ -1847,7 +1845,7 @@
         <v>98</v>
       </c>
       <c r="G19" t="s">
-        <v>118</v>
+        <v>136</v>
       </c>
       <c r="K19" s="1"/>
     </row>
@@ -1859,7 +1857,7 @@
         <v>98</v>
       </c>
       <c r="G20" t="s">
-        <v>119</v>
+        <v>137</v>
       </c>
       <c r="J20" s="1"/>
       <c r="K20" s="1"/>
@@ -1872,7 +1870,7 @@
         <v>98</v>
       </c>
       <c r="G21" t="s">
-        <v>120</v>
+        <v>138</v>
       </c>
       <c r="K21" s="1"/>
     </row>
@@ -1884,7 +1882,7 @@
         <v>98</v>
       </c>
       <c r="G22" t="s">
-        <v>121</v>
+        <v>139</v>
       </c>
       <c r="K22" s="1"/>
     </row>
@@ -1896,7 +1894,7 @@
         <v>98</v>
       </c>
       <c r="G23" t="s">
-        <v>122</v>
+        <v>140</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.3">
@@ -1907,7 +1905,7 @@
         <v>98</v>
       </c>
       <c r="G24" t="s">
-        <v>123</v>
+        <v>141</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.3">
@@ -1918,7 +1916,7 @@
         <v>98</v>
       </c>
       <c r="G25" t="s">
-        <v>124</v>
+        <v>142</v>
       </c>
       <c r="K25" s="1"/>
     </row>
@@ -1930,7 +1928,7 @@
         <v>98</v>
       </c>
       <c r="G26" t="s">
-        <v>125</v>
+        <v>143</v>
       </c>
       <c r="K26" s="1"/>
     </row>
@@ -1942,7 +1940,7 @@
         <v>98</v>
       </c>
       <c r="G27" t="s">
-        <v>126</v>
+        <v>144</v>
       </c>
       <c r="K27" s="1"/>
     </row>
@@ -1954,7 +1952,7 @@
         <v>99</v>
       </c>
       <c r="G28" t="s">
-        <v>127</v>
+        <v>145</v>
       </c>
       <c r="J28" s="1"/>
     </row>
@@ -1966,7 +1964,7 @@
         <v>99</v>
       </c>
       <c r="G29" t="s">
-        <v>128</v>
+        <v>146</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.3">
@@ -1977,7 +1975,7 @@
         <v>99</v>
       </c>
       <c r="G30" t="s">
-        <v>129</v>
+        <v>147</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.3">
@@ -1988,7 +1986,7 @@
         <v>99</v>
       </c>
       <c r="G31" t="s">
-        <v>130</v>
+        <v>148</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.3">
@@ -1999,7 +1997,7 @@
         <v>99</v>
       </c>
       <c r="G32" t="s">
-        <v>131</v>
+        <v>149</v>
       </c>
       <c r="J32" s="1"/>
     </row>
@@ -2011,7 +2009,7 @@
         <v>99</v>
       </c>
       <c r="G33" t="s">
-        <v>132</v>
+        <v>150</v>
       </c>
       <c r="K33" s="1"/>
     </row>
@@ -2023,7 +2021,7 @@
         <v>99</v>
       </c>
       <c r="G34" t="s">
-        <v>133</v>
+        <v>151</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.3">
@@ -2034,7 +2032,7 @@
         <v>99</v>
       </c>
       <c r="G35" t="s">
-        <v>134</v>
+        <v>152</v>
       </c>
       <c r="K35" s="1"/>
     </row>
@@ -2046,7 +2044,7 @@
         <v>99</v>
       </c>
       <c r="G36" t="s">
-        <v>135</v>
+        <v>153</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.3">
@@ -2057,7 +2055,7 @@
         <v>99</v>
       </c>
       <c r="G37" t="s">
-        <v>136</v>
+        <v>154</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.3">
@@ -2068,7 +2066,7 @@
         <v>99</v>
       </c>
       <c r="G38" t="s">
-        <v>137</v>
+        <v>155</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.3">
@@ -2079,7 +2077,7 @@
         <v>99</v>
       </c>
       <c r="G39" t="s">
-        <v>138</v>
+        <v>156</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.3">
@@ -2090,7 +2088,7 @@
         <v>99</v>
       </c>
       <c r="G40" t="s">
-        <v>139</v>
+        <v>157</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.3">
@@ -2101,7 +2099,7 @@
         <v>99</v>
       </c>
       <c r="G41" t="s">
-        <v>140</v>
+        <v>158</v>
       </c>
       <c r="K41" s="1"/>
     </row>
@@ -2113,7 +2111,7 @@
         <v>99</v>
       </c>
       <c r="G42" t="s">
-        <v>141</v>
+        <v>159</v>
       </c>
       <c r="K42" s="1"/>
     </row>
@@ -2125,7 +2123,7 @@
         <v>99</v>
       </c>
       <c r="G43" t="s">
-        <v>142</v>
+        <v>160</v>
       </c>
       <c r="K43" s="1"/>
     </row>
@@ -2137,7 +2135,7 @@
         <v>99</v>
       </c>
       <c r="G44" t="s">
-        <v>143</v>
+        <v>161</v>
       </c>
       <c r="K44" s="1"/>
     </row>
@@ -2149,7 +2147,7 @@
         <v>99</v>
       </c>
       <c r="G45" t="s">
-        <v>144</v>
+        <v>162</v>
       </c>
       <c r="K45" s="1"/>
     </row>
@@ -2161,7 +2159,7 @@
         <v>99</v>
       </c>
       <c r="G46" t="s">
-        <v>145</v>
+        <v>163</v>
       </c>
       <c r="J46" s="1"/>
     </row>
@@ -2173,7 +2171,7 @@
         <v>99</v>
       </c>
       <c r="G47" t="s">
-        <v>146</v>
+        <v>164</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.3">
@@ -2184,7 +2182,7 @@
         <v>99</v>
       </c>
       <c r="G48" t="s">
-        <v>147</v>
+        <v>165</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.3">
@@ -2195,7 +2193,7 @@
         <v>99</v>
       </c>
       <c r="G49" t="s">
-        <v>148</v>
+        <v>166</v>
       </c>
       <c r="K49" s="1"/>
     </row>
@@ -2207,7 +2205,7 @@
         <v>99</v>
       </c>
       <c r="G50" t="s">
-        <v>149</v>
+        <v>167</v>
       </c>
       <c r="K50" s="1"/>
     </row>
@@ -2219,7 +2217,7 @@
         <v>99</v>
       </c>
       <c r="G51" t="s">
-        <v>150</v>
+        <v>168</v>
       </c>
       <c r="K51" s="1"/>
     </row>
@@ -2231,7 +2229,7 @@
         <v>99</v>
       </c>
       <c r="G52" t="s">
-        <v>151</v>
+        <v>169</v>
       </c>
       <c r="K52" s="1"/>
     </row>
@@ -2243,7 +2241,7 @@
         <v>99</v>
       </c>
       <c r="G53" t="s">
-        <v>152</v>
+        <v>170</v>
       </c>
       <c r="K53" s="1"/>
     </row>
@@ -2255,7 +2253,7 @@
         <v>99</v>
       </c>
       <c r="G54" t="s">
-        <v>153</v>
+        <v>171</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.3">
@@ -2266,7 +2264,7 @@
         <v>99</v>
       </c>
       <c r="G55" t="s">
-        <v>154</v>
+        <v>172</v>
       </c>
       <c r="K55" s="1"/>
     </row>
@@ -2278,7 +2276,7 @@
         <v>99</v>
       </c>
       <c r="G56" t="s">
-        <v>155</v>
+        <v>173</v>
       </c>
       <c r="K56" s="1"/>
     </row>
@@ -2290,7 +2288,7 @@
         <v>99</v>
       </c>
       <c r="G57" t="s">
-        <v>156</v>
+        <v>174</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.3">
@@ -2301,7 +2299,7 @@
         <v>99</v>
       </c>
       <c r="G58" t="s">
-        <v>157</v>
+        <v>175</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.3">
@@ -2312,7 +2310,7 @@
         <v>100</v>
       </c>
       <c r="G59" t="s">
-        <v>158</v>
+        <v>176</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.3">
@@ -2323,7 +2321,7 @@
         <v>100</v>
       </c>
       <c r="G60" t="s">
-        <v>159</v>
+        <v>177</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.3">
@@ -2334,7 +2332,7 @@
         <v>100</v>
       </c>
       <c r="G61" t="s">
-        <v>160</v>
+        <v>178</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.3">
@@ -2345,7 +2343,7 @@
         <v>100</v>
       </c>
       <c r="G62" t="s">
-        <v>161</v>
+        <v>179</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.3">
@@ -2356,7 +2354,7 @@
         <v>100</v>
       </c>
       <c r="G63" t="s">
-        <v>162</v>
+        <v>180</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.3">
@@ -2367,7 +2365,7 @@
         <v>100</v>
       </c>
       <c r="G64" t="s">
-        <v>163</v>
+        <v>181</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.3">
@@ -2378,7 +2376,7 @@
         <v>100</v>
       </c>
       <c r="G65" t="s">
-        <v>164</v>
+        <v>182</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.3">
@@ -2389,7 +2387,7 @@
         <v>100</v>
       </c>
       <c r="G66" t="s">
-        <v>165</v>
+        <v>183</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.3">
@@ -2400,7 +2398,7 @@
         <v>100</v>
       </c>
       <c r="G67" t="s">
-        <v>166</v>
+        <v>184</v>
       </c>
       <c r="K67" s="1"/>
     </row>
@@ -2412,7 +2410,7 @@
         <v>100</v>
       </c>
       <c r="G68" t="s">
-        <v>167</v>
+        <v>185</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.3">
@@ -2423,7 +2421,7 @@
         <v>100</v>
       </c>
       <c r="G69" t="s">
-        <v>168</v>
+        <v>186</v>
       </c>
       <c r="J69" s="1"/>
       <c r="K69" s="1"/>
@@ -2436,7 +2434,7 @@
         <v>100</v>
       </c>
       <c r="G70" t="s">
-        <v>169</v>
+        <v>187</v>
       </c>
       <c r="K70" s="1"/>
     </row>
@@ -2448,7 +2446,7 @@
         <v>100</v>
       </c>
       <c r="G71" t="s">
-        <v>170</v>
+        <v>188</v>
       </c>
       <c r="J71" s="1"/>
       <c r="K71" s="1"/>
@@ -2461,7 +2459,7 @@
         <v>100</v>
       </c>
       <c r="G72" t="s">
-        <v>171</v>
+        <v>189</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.3">
@@ -2472,7 +2470,7 @@
         <v>100</v>
       </c>
       <c r="G73" t="s">
-        <v>172</v>
+        <v>190</v>
       </c>
       <c r="K73" s="1"/>
     </row>
@@ -2484,7 +2482,7 @@
         <v>100</v>
       </c>
       <c r="G74" t="s">
-        <v>173</v>
+        <v>191</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.3">
@@ -2495,7 +2493,7 @@
         <v>100</v>
       </c>
       <c r="G75" t="s">
-        <v>174</v>
+        <v>192</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.3">
@@ -2506,7 +2504,7 @@
         <v>100</v>
       </c>
       <c r="G76" t="s">
-        <v>175</v>
+        <v>193</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.3">
@@ -2517,7 +2515,7 @@
         <v>100</v>
       </c>
       <c r="G77" t="s">
-        <v>176</v>
+        <v>194</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.3">
@@ -2528,7 +2526,7 @@
         <v>100</v>
       </c>
       <c r="G78" t="s">
-        <v>177</v>
+        <v>195</v>
       </c>
       <c r="K78" s="1"/>
     </row>
@@ -2540,7 +2538,7 @@
         <v>100</v>
       </c>
       <c r="G79" t="s">
-        <v>178</v>
+        <v>196</v>
       </c>
       <c r="K79" s="1"/>
     </row>
@@ -2552,7 +2550,7 @@
         <v>100</v>
       </c>
       <c r="G80" t="s">
-        <v>179</v>
+        <v>197</v>
       </c>
       <c r="K80" s="1"/>
     </row>
@@ -2564,7 +2562,7 @@
         <v>100</v>
       </c>
       <c r="G81" t="s">
-        <v>180</v>
+        <v>198</v>
       </c>
       <c r="K81" s="1"/>
     </row>
@@ -2576,16 +2574,16 @@
         <v>100</v>
       </c>
       <c r="G82" t="s">
-        <v>181</v>
+        <v>199</v>
       </c>
       <c r="K82" s="1"/>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A83" s="3" t="s">
-        <v>182</v>
+        <v>101</v>
       </c>
       <c r="B83" t="s">
-        <v>199</v>
+        <v>118</v>
       </c>
       <c r="G83" t="s">
         <v>200</v>
@@ -2594,10 +2592,10 @@
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A84" s="3" t="s">
-        <v>183</v>
+        <v>102</v>
       </c>
       <c r="B84" t="s">
-        <v>199</v>
+        <v>118</v>
       </c>
       <c r="G84" t="s">
         <v>201</v>
@@ -2606,10 +2604,10 @@
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A85" s="3" t="s">
-        <v>184</v>
+        <v>103</v>
       </c>
       <c r="B85" t="s">
-        <v>199</v>
+        <v>118</v>
       </c>
       <c r="G85" t="s">
         <v>202</v>
@@ -2618,10 +2616,10 @@
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A86" s="3" t="s">
-        <v>185</v>
+        <v>104</v>
       </c>
       <c r="B86" t="s">
-        <v>199</v>
+        <v>118</v>
       </c>
       <c r="G86" t="s">
         <v>203</v>
@@ -2630,10 +2628,10 @@
     </row>
     <row r="87" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A87" s="3" t="s">
-        <v>186</v>
+        <v>105</v>
       </c>
       <c r="B87" t="s">
-        <v>199</v>
+        <v>118</v>
       </c>
       <c r="G87" t="s">
         <v>204</v>
@@ -2642,10 +2640,10 @@
     </row>
     <row r="88" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A88" s="3" t="s">
-        <v>187</v>
+        <v>106</v>
       </c>
       <c r="B88" t="s">
-        <v>199</v>
+        <v>118</v>
       </c>
       <c r="G88" t="s">
         <v>205</v>
@@ -2654,10 +2652,10 @@
     </row>
     <row r="89" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A89" s="3" t="s">
-        <v>188</v>
+        <v>107</v>
       </c>
       <c r="B89" t="s">
-        <v>199</v>
+        <v>118</v>
       </c>
       <c r="G89" t="s">
         <v>206</v>
@@ -2666,10 +2664,10 @@
     </row>
     <row r="90" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A90" s="3" t="s">
-        <v>189</v>
+        <v>108</v>
       </c>
       <c r="B90" t="s">
-        <v>199</v>
+        <v>118</v>
       </c>
       <c r="G90" t="s">
         <v>207</v>
@@ -2678,10 +2676,10 @@
     </row>
     <row r="91" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A91" s="3" t="s">
-        <v>190</v>
+        <v>109</v>
       </c>
       <c r="B91" t="s">
-        <v>199</v>
+        <v>118</v>
       </c>
       <c r="G91" t="s">
         <v>208</v>
@@ -2690,10 +2688,10 @@
     </row>
     <row r="92" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A92" s="3" t="s">
-        <v>191</v>
+        <v>110</v>
       </c>
       <c r="B92" t="s">
-        <v>199</v>
+        <v>118</v>
       </c>
       <c r="F92" s="2"/>
       <c r="G92" t="s">
@@ -2703,10 +2701,10 @@
     </row>
     <row r="93" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A93" s="3" t="s">
-        <v>192</v>
+        <v>111</v>
       </c>
       <c r="B93" t="s">
-        <v>199</v>
+        <v>118</v>
       </c>
       <c r="G93" t="s">
         <v>210</v>
@@ -2715,10 +2713,10 @@
     </row>
     <row r="94" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A94" s="3" t="s">
-        <v>193</v>
+        <v>112</v>
       </c>
       <c r="B94" t="s">
-        <v>199</v>
+        <v>118</v>
       </c>
       <c r="G94" t="s">
         <v>211</v>
@@ -2727,10 +2725,10 @@
     </row>
     <row r="95" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A95" s="3" t="s">
-        <v>194</v>
+        <v>113</v>
       </c>
       <c r="B95" t="s">
-        <v>199</v>
+        <v>118</v>
       </c>
       <c r="G95" t="s">
         <v>202</v>
@@ -2739,10 +2737,10 @@
     </row>
     <row r="96" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A96" s="3" t="s">
-        <v>195</v>
+        <v>114</v>
       </c>
       <c r="B96" t="s">
-        <v>199</v>
+        <v>118</v>
       </c>
       <c r="G96" t="s">
         <v>212</v>
@@ -2751,10 +2749,10 @@
     </row>
     <row r="97" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A97" s="3" t="s">
-        <v>196</v>
+        <v>115</v>
       </c>
       <c r="B97" t="s">
-        <v>199</v>
+        <v>118</v>
       </c>
       <c r="G97" t="s">
         <v>213</v>
@@ -2763,10 +2761,10 @@
     </row>
     <row r="98" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A98" s="3" t="s">
-        <v>197</v>
+        <v>116</v>
       </c>
       <c r="B98" t="s">
-        <v>199</v>
+        <v>118</v>
       </c>
       <c r="G98" t="s">
         <v>214</v>
@@ -2775,10 +2773,10 @@
     </row>
     <row r="99" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A99" s="3" t="s">
-        <v>198</v>
+        <v>117</v>
       </c>
       <c r="B99" t="s">
-        <v>199</v>
+        <v>118</v>
       </c>
       <c r="G99" t="s">
         <v>215</v>
@@ -2794,8 +2792,8 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101001758D32B18DD85479881024DF1B1560C" ma:contentTypeVersion="24" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="81ef2f892c483f306f0558c148ab3d80">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="67842d5e-ae6d-4c89-a872-a2ee0755ec95" xmlns:ns3="a1875003-4be3-4a6e-8a8c-096c5e566ae9" xmlns:ns4="da4bd983-6116-4324-b7f3-01d16dca807e" xmlns:ns5="aede6c6b-3004-496c-ae85-a12871320d3d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e20b0ceab88938c995cc17af9cada473" ns1:_="" ns2:_="" ns3:_="" ns4:_="" ns5:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101001758D32B18DD85479881024DF1B1560C" ma:contentTypeVersion="24" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="17c547b8ab5b97348d139d0b9b91e586">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="67842d5e-ae6d-4c89-a872-a2ee0755ec95" xmlns:ns3="a1875003-4be3-4a6e-8a8c-096c5e566ae9" xmlns:ns4="da4bd983-6116-4324-b7f3-01d16dca807e" xmlns:ns5="aede6c6b-3004-496c-ae85-a12871320d3d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="068ac477613bd444312304782eaa7631" ns1:_="" ns2:_="" ns3:_="" ns4:_="" ns5:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
     <xsd:import namespace="67842d5e-ae6d-4c89-a872-a2ee0755ec95"/>
     <xsd:import namespace="a1875003-4be3-4a6e-8a8c-096c5e566ae9"/>
@@ -2909,7 +2907,7 @@
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="a1875003-4be3-4a6e-8a8c-096c5e566ae9" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="11" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de imagen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="8d84b6a1-61d2-4825-be3a-9ba6e50d6236" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="11" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="8d84b6a1-61d2-4825-be3a-9ba6e50d6236" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
       <xsd:complexType>
         <xsd:sequence>
           <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
@@ -2971,8 +2969,8 @@
         <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de contenido"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
         <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
         <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
@@ -3062,15 +3060,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
@@ -3083,14 +3072,35 @@
 </p:properties>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8D515F7C-5746-484F-B078-B8A910ECCF08}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED1BFC5A-8E78-46F6-9523-69B548367BD1}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C9516AC-4061-4301-AD48-5779E805CF9C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AD97F44E-6559-4391-9A6B-710EF331E17C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="aede6c6b-3004-496c-ae85-a12871320d3d"/>
+    <ds:schemaRef ds:uri="a1875003-4be3-4a6e-8a8c-096c5e566ae9"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AD97F44E-6559-4391-9A6B-710EF331E17C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C9516AC-4061-4301-AD48-5779E805CF9C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>